<commit_message>
Historique KPI — 18/09/2026
</commit_message>
<xml_diff>
--- a/kpis/indicateurs_kpis.xlsx
+++ b/kpis/indicateurs_kpis.xlsx
@@ -7469,7 +7469,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>92.31</t>
         </is>
       </c>
     </row>
@@ -7546,7 +7546,7 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>92.31</t>
         </is>
       </c>
     </row>
@@ -7623,7 +7623,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>92.31</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7854,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>84.62</t>
         </is>
       </c>
     </row>
@@ -8132,17 +8132,17 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>96.2</t>
+          <t>79.4</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>2.9</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>17.6</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -8162,7 +8162,7 @@
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>84.62</t>
+          <t>69.23</t>
         </is>
       </c>
     </row>
@@ -9672,17 +9672,17 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>99.0</t>
+          <t>99.3</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
@@ -9818,7 +9818,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>0</v>
@@ -9836,7 +9836,7 @@
         <v>36</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38">
@@ -9867,7 +9867,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>0</v>
@@ -9885,7 +9885,7 @@
         <v>7</v>
       </c>
       <c r="O38" s="3" t="n">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="39">
@@ -9916,7 +9916,7 @@
         <v>0</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" s="3" t="n">
         <v>0</v>
@@ -9934,7 +9934,7 @@
         <v>15</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="40">
@@ -9965,7 +9965,7 @@
         <v>0</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J40" s="3" t="n">
         <v>0</v>
@@ -9983,7 +9983,7 @@
         <v>3</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41">
@@ -10014,7 +10014,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J41" s="3" t="n">
         <v>0</v>
@@ -10032,7 +10032,7 @@
         <v>1</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="42">
@@ -10161,25 +10161,25 @@
         <v>0</v>
       </c>
       <c r="I44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="3" t="n">
         <v>3</v>
-      </c>
-      <c r="J44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" s="3" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -10210,25 +10210,25 @@
         <v>0</v>
       </c>
       <c r="I45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="3" t="n">
         <v>1</v>
-      </c>
-      <c r="J45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" s="3" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -10259,7 +10259,7 @@
         <v>0</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J46" s="3" t="n">
         <v>0</v>
@@ -10277,7 +10277,7 @@
         <v>1</v>
       </c>
       <c r="O46" s="3" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47">
@@ -10290,13 +10290,13 @@
         <v>26</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" s="3" t="n">
         <v>0</v>
@@ -10308,13 +10308,13 @@
         <v>0</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="J47" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L47" s="3" t="n">
         <v>0</v>
@@ -10326,7 +10326,7 @@
         <v>8</v>
       </c>
       <c r="O47" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48">
@@ -10406,25 +10406,25 @@
         <v>0</v>
       </c>
       <c r="I49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="3" t="n">
         <v>4</v>
-      </c>
-      <c r="J49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O49" s="3" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -10553,7 +10553,7 @@
         <v>0</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J52" s="3" t="n">
         <v>0</v>
@@ -10571,7 +10571,7 @@
         <v>14</v>
       </c>
       <c r="O52" s="3" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53">
@@ -10602,25 +10602,25 @@
         <v>0</v>
       </c>
       <c r="I53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="3" t="n">
         <v>10</v>
-      </c>
-      <c r="J53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O53" s="3" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="54">
@@ -10651,25 +10651,25 @@
         <v>0</v>
       </c>
       <c r="I54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="J54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="3" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="55">
@@ -10700,7 +10700,7 @@
         <v>0</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J55" s="3" t="n">
         <v>0</v>
@@ -10718,7 +10718,7 @@
         <v>0</v>
       </c>
       <c r="O55" s="3" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="56">
@@ -11221,13 +11221,13 @@
         <v>107</v>
       </c>
       <c r="C66" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D66" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>0</v>
@@ -11239,13 +11239,13 @@
         <v>0</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>91</v>
+        <v>7</v>
       </c>
       <c r="J66" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L66" s="3" t="n">
         <v>0</v>
@@ -11257,7 +11257,7 @@
         <v>111</v>
       </c>
       <c r="O66" s="3" t="n">
-        <v>1135</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="68">
@@ -11367,7 +11367,7 @@
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11404,7 +11404,7 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>98.6</t>
+          <t>99.3</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11471,7 +11471,7 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>97.3</t>
+          <t>98.4</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11575,7 +11575,7 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11627,7 +11627,7 @@
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11691,7 +11691,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -11758,7 +11758,7 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -11768,7 +11768,7 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>98.5</t>
+          <t>99.7</t>
         </is>
       </c>
       <c r="H78" s="3" t="inlineStr">
@@ -11783,7 +11783,7 @@
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>75.00</t>
         </is>
       </c>
     </row>
@@ -11835,7 +11835,7 @@
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -11847,7 +11847,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -11862,7 +11862,7 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>87.50</t>
+          <t>75.00</t>
         </is>
       </c>
     </row>
@@ -11914,7 +11914,7 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -11939,7 +11939,7 @@
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>75.00</t>
         </is>
       </c>
     </row>
@@ -11966,7 +11966,7 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>75.00</t>
         </is>
       </c>
     </row>
@@ -12043,7 +12043,7 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12095,7 +12095,7 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12107,7 +12107,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -12251,7 +12251,7 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12288,7 +12288,7 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>97.0</t>
+          <t>97.2</t>
         </is>
       </c>
       <c r="H88" s="3" t="inlineStr">
@@ -12303,7 +12303,7 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12340,7 +12340,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>96.8</t>
+          <t>97.1</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
@@ -12355,7 +12355,7 @@
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12407,7 +12407,7 @@
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12459,7 +12459,7 @@
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12563,7 +12563,7 @@
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12615,7 +12615,7 @@
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12667,7 +12667,7 @@
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12719,7 +12719,7 @@
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12771,7 +12771,7 @@
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12823,7 +12823,7 @@
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>87.50</t>
         </is>
       </c>
     </row>
@@ -12887,7 +12887,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -12902,7 +12902,7 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>99.5</t>
+          <t>99.6</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
@@ -12927,7 +12927,7 @@
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>87.50</t>
+          <t>75.00</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13046,7 @@
         <v>0</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H105" s="3" t="n">
         <v>0</v>
@@ -13055,7 +13055,7 @@
         <v>0</v>
       </c>
       <c r="J105" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -13114,7 +13114,7 @@
         <v>0</v>
       </c>
       <c r="G107" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H107" s="3" t="n">
         <v>0</v>
@@ -13123,7 +13123,7 @@
         <v>0</v>
       </c>
       <c r="J107" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="108">
@@ -13278,13 +13278,13 @@
         <v>0</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F112" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G112" s="3" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="H112" s="3" t="n">
         <v>0</v>
@@ -13293,7 +13293,7 @@
         <v>0</v>
       </c>
       <c r="J112" s="3" t="n">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="113">
@@ -13318,7 +13318,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H113" s="3" t="n">
         <v>0</v>
@@ -13327,7 +13327,7 @@
         <v>0</v>
       </c>
       <c r="J113" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -13346,7 +13346,7 @@
         <v>0</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F114" s="3" t="n">
         <v>0</v>
@@ -13361,7 +13361,7 @@
         <v>0</v>
       </c>
       <c r="J114" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115">
@@ -13380,7 +13380,7 @@
         <v>0</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F115" s="3" t="n">
         <v>0</v>
@@ -13395,7 +13395,7 @@
         <v>0</v>
       </c>
       <c r="J115" s="3" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="116">
@@ -13414,7 +13414,7 @@
         <v>0</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F116" s="3" t="n">
         <v>0</v>
@@ -13429,7 +13429,7 @@
         <v>0</v>
       </c>
       <c r="J116" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117">
@@ -13624,7 +13624,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H122" s="3" t="n">
         <v>0</v>
@@ -13633,7 +13633,7 @@
         <v>0</v>
       </c>
       <c r="J122" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123">
@@ -13658,16 +13658,16 @@
         <v>1</v>
       </c>
       <c r="G123" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H123" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J123" s="3" t="n">
         <v>10</v>
-      </c>
-      <c r="H123" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I123" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J123" s="3" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="124">
@@ -13992,13 +13992,13 @@
         <v>0</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F133" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G133" s="3" t="n">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="H133" s="3" t="n">
         <v>0</v>
@@ -14007,7 +14007,7 @@
         <v>0</v>
       </c>
       <c r="J133" s="3" t="n">
-        <v>187</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Historique KPI — 25/09/2026
</commit_message>
<xml_diff>
--- a/kpis/indicateurs_kpis.xlsx
+++ b/kpis/indicateurs_kpis.xlsx
@@ -21573,7 +21573,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>99.6</t>
+          <t>99.3</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>99.7</t>
+          <t>99.5</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -22221,7 +22221,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -22231,7 +22231,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -22281,7 +22281,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>84.62</t>
         </is>
       </c>
     </row>
@@ -23222,7 +23222,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>96.6</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -23232,7 +23232,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>96.6</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -23282,7 +23282,7 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>99.47</t>
         </is>
       </c>
     </row>
@@ -23398,7 +23398,7 @@
         <v>0</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="J37" s="3" t="n">
         <v>0</v>
@@ -23416,7 +23416,7 @@
         <v>4</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38">
@@ -23790,7 +23790,7 @@
         <v>0</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="J45" s="3" t="n">
         <v>0</v>
@@ -23799,7 +23799,7 @@
         <v>0</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="M45" s="3" t="n">
         <v>0</v>
@@ -23808,7 +23808,7 @@
         <v>0</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>60</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46">
@@ -23937,7 +23937,7 @@
         <v>0</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="J48" s="3" t="n">
         <v>0</v>
@@ -23946,7 +23946,7 @@
         <v>0</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M48" s="3" t="n">
         <v>0</v>
@@ -23955,7 +23955,7 @@
         <v>0</v>
       </c>
       <c r="O48" s="3" t="n">
-        <v>34</v>
+        <v>55</v>
       </c>
     </row>
     <row r="49">
@@ -23986,7 +23986,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="J49" s="3" t="n">
         <v>0</v>
@@ -24004,7 +24004,7 @@
         <v>0</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>11</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50">
@@ -24219,7 +24219,7 @@
         <v>0</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>0</v>
@@ -24249,7 +24249,7 @@
         <v>0</v>
       </c>
       <c r="O54" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -24427,7 +24427,7 @@
         <v>0</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="J58" s="3" t="n">
         <v>0</v>
@@ -24445,7 +24445,7 @@
         <v>4</v>
       </c>
       <c r="O58" s="3" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
     </row>
     <row r="59">
@@ -24770,7 +24770,7 @@
         <v>0</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J65" s="3" t="n">
         <v>0</v>
@@ -24788,7 +24788,7 @@
         <v>0</v>
       </c>
       <c r="O65" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66">
@@ -24807,7 +24807,7 @@
         <v>0</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F66" s="3" t="n">
         <v>17</v>
@@ -24819,7 +24819,7 @@
         <v>0</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>162</v>
+        <v>293</v>
       </c>
       <c r="J66" s="3" t="n">
         <v>0</v>
@@ -24828,7 +24828,7 @@
         <v>0</v>
       </c>
       <c r="L66" s="3" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="M66" s="3" t="n">
         <v>24</v>
@@ -24837,7 +24837,7 @@
         <v>27</v>
       </c>
       <c r="O66" s="3" t="n">
-        <v>306</v>
+        <v>454</v>
       </c>
     </row>
     <row r="68">

</xml_diff>